<commit_message>
feat: add auto start chrome
</commit_message>
<xml_diff>
--- a/input/点赞_用户列表.xlsx
+++ b/input/点赞_用户列表.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B513"/>
+  <dimension ref="A1:B552"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -572,7 +572,7 @@
         <v>麤麤酱二次元</v>
       </c>
       <c r="B22" t="str">
-        <v>2026-01-20</v>
+        <v>2026-03-23</v>
       </c>
     </row>
     <row r="23">
@@ -1636,7 +1636,7 @@
         <v>CC妙脆角</v>
       </c>
       <c r="B155" t="str">
-        <v>2026-01-14</v>
+        <v>2026-03-23</v>
       </c>
     </row>
     <row r="156">
@@ -2068,7 +2068,7 @@
         <v>莫言會拍照</v>
       </c>
       <c r="B209" t="str">
-        <v>2026-01-13</v>
+        <v>2026-03-23</v>
       </c>
     </row>
     <row r="210">
@@ -2116,7 +2116,7 @@
         <v>小艾解忧铺</v>
       </c>
       <c r="B215" t="str">
-        <v>2026-01-18</v>
+        <v>2026-03-23</v>
       </c>
     </row>
     <row r="216">
@@ -2820,7 +2820,7 @@
         <v>挪威唱民歌的芝士</v>
       </c>
       <c r="B303" t="str">
-        <v>2026-02-06</v>
+        <v>2026-03-23</v>
       </c>
     </row>
     <row r="304">
@@ -3020,7 +3020,7 @@
         <v>娜娜是我呀</v>
       </c>
       <c r="B328" t="str">
-        <v>2026-01-18</v>
+        <v>2026-03-23</v>
       </c>
     </row>
     <row r="329">
@@ -3212,7 +3212,7 @@
         <v>小桔子家电批发</v>
       </c>
       <c r="B352" t="str">
-        <v>2026-01-20</v>
+        <v>2026-03-23</v>
       </c>
     </row>
     <row r="353">
@@ -3436,7 +3436,7 @@
         <v>淡淡的咸鱼</v>
       </c>
       <c r="B380" t="str">
-        <v>2026-01-17</v>
+        <v>2026-03-23</v>
       </c>
     </row>
     <row r="381">
@@ -3812,7 +3812,7 @@
         <v>娜娜的口袋</v>
       </c>
       <c r="B427" t="str">
-        <v>2026-01-18</v>
+        <v>2026-03-23</v>
       </c>
     </row>
     <row r="428">
@@ -4236,7 +4236,7 @@
         <v>暖家优选小家电</v>
       </c>
       <c r="B480" t="str">
-        <v>2026-02-06</v>
+        <v>2026-03-23</v>
       </c>
     </row>
     <row r="481">
@@ -4324,7 +4324,7 @@
         <v>强者资源库</v>
       </c>
       <c r="B491" t="str">
-        <v>2026-02-06</v>
+        <v>2026-03-23</v>
       </c>
     </row>
     <row r="492">
@@ -4503,9 +4503,321 @@
         <v>2026-02-06</v>
       </c>
     </row>
+    <row r="514">
+      <c r="A514" t="str">
+        <v>柠源优品</v>
+      </c>
+      <c r="B514" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="str">
+        <v>甜净生活馆</v>
+      </c>
+      <c r="B515" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="str">
+        <v>壹人小家电</v>
+      </c>
+      <c r="B516" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="str">
+        <v>橘子味的秋天</v>
+      </c>
+      <c r="B517" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="str">
+        <v>品质家电严选店</v>
+      </c>
+      <c r="B518" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="str">
+        <v>小杨数码科技</v>
+      </c>
+      <c r="B519" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="str">
+        <v>智享科技</v>
+      </c>
+      <c r="B520" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="str">
+        <v>伊伊家电</v>
+      </c>
+      <c r="B521" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="str">
+        <v>羽球小哥的二手球</v>
+      </c>
+      <c r="B522" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="str">
+        <v>小云严选数码</v>
+      </c>
+      <c r="B523" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="str">
+        <v>狸狸次元屋</v>
+      </c>
+      <c r="B524" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="str">
+        <v>毛毛的玩偶屋</v>
+      </c>
+      <c r="B525" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="str">
+        <v>G小王子</v>
+      </c>
+      <c r="B526" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="str">
+        <v>小枝百货铺</v>
+      </c>
+      <c r="B527" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="str">
+        <v>大鱼和小余店铺</v>
+      </c>
+      <c r="B528" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="str">
+        <v>布偶猫的百宝袋</v>
+      </c>
+      <c r="B529" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="str">
+        <v>乐乐严选家电</v>
+      </c>
+      <c r="B530" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="str">
+        <v>小E的宝藏清单</v>
+      </c>
+      <c r="B531" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="str">
+        <v>美术馆会玩的翻车鱼</v>
+      </c>
+      <c r="B532" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="str">
+        <v>诚品数码铺</v>
+      </c>
+      <c r="B533" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="str">
+        <v/>
+      </c>
+      <c r="B534" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="str">
+        <v>海伦的小店铺</v>
+      </c>
+      <c r="B535" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="str">
+        <v>快乐小宝</v>
+      </c>
+      <c r="B536" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="str">
+        <v>六一小仙女呀</v>
+      </c>
+      <c r="B537" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="str">
+        <v>佳忱杂货屋</v>
+      </c>
+      <c r="B538" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="str">
+        <v>小叮当猫</v>
+      </c>
+      <c r="B539" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="str">
+        <v>科研猎人</v>
+      </c>
+      <c r="B540" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="str">
+        <v>百宝箱杂货铺</v>
+      </c>
+      <c r="B541" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="str">
+        <v>是小鱼儿</v>
+      </c>
+      <c r="B542" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="str">
+        <v>虫乃的周边小铺</v>
+      </c>
+      <c r="B543" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="str">
+        <v>优选好品质家电馆</v>
+      </c>
+      <c r="B544" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="str">
+        <v>小馋猫家卡券</v>
+      </c>
+      <c r="B545" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="str">
+        <v>拾光家选</v>
+      </c>
+      <c r="B546" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="str">
+        <v>零下一度</v>
+      </c>
+      <c r="B547" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="str">
+        <v>鱼鱼的小铺</v>
+      </c>
+      <c r="B548" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="str">
+        <v>花生老板不卖花生</v>
+      </c>
+      <c r="B549" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="str">
+        <v>正品小家电</v>
+      </c>
+      <c r="B550" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="str">
+        <v>小黎的拆盒铺</v>
+      </c>
+      <c r="B551" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="str">
+        <v>时尚包包好看嘛</v>
+      </c>
+      <c r="B552" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B513"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B552"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>